<commit_message>
correcao nos ultimos testes
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1250_40/resumo_consolidado_com_MI.xlsx
+++ b/alocacao/saidas_1250_40/resumo_consolidado_com_MI.xlsx
@@ -539,14 +539,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>abastecimento_10wlim_1250</t>
+          <t>abastecimento_full_1250</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>17602</v>
+        <v>17271</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>77</v>
+        <v>370</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -554,34 +554,34 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>953429.11</v>
+        <v>977683.91</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>990039.77</v>
+        <v>1071061.64</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>1350401.97</v>
+        <v>1482780.51</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" s="4" t="n">
-        <v>41.64</v>
+        <v>51.66</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>3.84</v>
+        <v>9.550000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>abastecimento_full_1250</t>
+          <t>abastecimento_limite_1250</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>16879</v>
+        <v>17106</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>402</v>
+        <v>301</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -589,34 +589,34 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>952888.8</v>
+        <v>979350.45</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1040361.88</v>
+        <v>1075945.57</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1410417.54</v>
+        <v>1482252.61</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" s="4" t="n">
-        <v>48.01</v>
+        <v>51.35</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>9.18</v>
+        <v>9.859999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>abastecimento_limite_1250</t>
+          <t>abastecimento_10wlim_1250</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>16724</v>
+        <v>17602</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>245</v>
+        <v>77</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -624,21 +624,21 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>941018.42</v>
+        <v>953429.11</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1041580.94</v>
+        <v>990056.72</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1418584.23</v>
+        <v>1350401.97</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" s="4" t="n">
-        <v>50.75</v>
+        <v>41.64</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>10.69</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="6">

</xml_diff>